<commit_message>
Add LLaVA-1.5-13B full results (baseline + BTP) + updated Excel
</commit_message>
<xml_diff>
--- a/BTP-Reproduction/BTP_Reproduction_Results.xlsx
+++ b/BTP-Reproduction/BTP_Reproduction_Results.xlsx
@@ -8,8 +8,9 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Results" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="LLaVA-1.5-7B" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Run Log" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="LLaVA-1.5-13B" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="49">
   <si>
     <t xml:space="preserve">BTP Reproduction — LLaVA-v1.5-7B</t>
   </si>
@@ -162,6 +163,12 @@
   </si>
   <si>
     <t xml:space="preserve">20260612_121210_results.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LLaVA-v1.5-13B — Paper vs Ours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IIT Jodhpur HPC, A100-40GB, FlashAttention-2, full datasets</t>
   </si>
 </sst>
 </file>
@@ -302,24 +309,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -327,7 +330,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -335,11 +338,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -596,266 +599,266 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>61.98</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="6" t="n">
         <f aca="false">C6-B6</f>
         <v>-0.0200000000000031</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="6" t="n">
         <v>1510.7</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>1507.5</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="6" t="n">
         <f aca="false">C7-B7</f>
         <v>-3.20000000000005</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="6" t="n">
         <v>64.3</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>64</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="6" t="n">
         <f aca="false">C8-B8</f>
         <v>-0.299999999999997</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="6" t="n">
         <v>85.8</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="6" t="n">
         <v>86.98</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="6" t="n">
         <f aca="false">C9-B9</f>
         <v>1.18000000000001</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="6" t="n">
         <v>69.4</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="6" t="n">
         <v>69.41</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="6" t="n">
         <f aca="false">C10-B10</f>
         <v>0.00999999999999091</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="6" t="n">
         <v>59</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="6" t="n">
         <v>58.98</v>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="6" t="n">
         <f aca="false">C14-B14</f>
         <v>-0.0200000000000031</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="6" t="n">
         <v>1487</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="6" t="n">
         <v>1497.2</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="6" t="n">
         <f aca="false">C15-B15</f>
         <v>10.2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="6" t="n">
         <v>62.7</v>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="6" t="n">
         <v>63.49</v>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="6" t="n">
         <f aca="false">C16-B16</f>
         <v>0.789999999999999</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="7" t="n">
+      <c r="B17" s="6" t="n">
         <v>85.6</v>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="6" t="n">
         <v>85.36</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="6" t="n">
         <f aca="false">C17-B17</f>
         <v>-0.239999999999995</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B18" s="6" t="n">
         <v>69.1</v>
       </c>
-      <c r="C18" s="7" t="n">
+      <c r="C18" s="6" t="n">
         <v>69.21</v>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D18" s="6" t="n">
         <f aca="false">C18-B18</f>
         <v>0.109999999999999</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="7" t="n">
+      <c r="B22" s="6" t="n">
         <v>46.11</v>
       </c>
-      <c r="C22" s="7" t="n">
+      <c r="C22" s="6" t="n">
         <v>40.02</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B23" s="7" t="n">
+      <c r="B23" s="6" t="n">
         <v>66.23</v>
       </c>
-      <c r="C23" s="7" t="n">
+      <c r="C23" s="6" t="n">
         <v>63.99</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="7" t="n">
+      <c r="B24" s="6" t="n">
         <v>355.7</v>
       </c>
-      <c r="C24" s="7" t="n">
+      <c r="C24" s="6" t="n">
         <v>351.4</v>
       </c>
     </row>
@@ -881,266 +884,266 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="7" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="n">
+      <c r="A2" s="8" t="n">
         <v>343354</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="9" t="n">
+      <c r="D2" s="8" t="n">
         <v>1028</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="n">
+      <c r="A3" s="8" t="n">
         <v>343354</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="9" t="n">
+      <c r="D3" s="8" t="n">
         <v>430</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="8" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="n">
+      <c r="A4" s="8" t="n">
         <v>343354</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="D4" s="8" t="n">
         <v>643</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="8" t="n">
         <v>343354</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="8" t="n">
         <v>1161</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="8" t="n">
         <v>343354</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="8" t="n">
         <v>2182</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="8" t="n">
         <v>343354</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>9510</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="n">
+      <c r="A8" s="8" t="n">
         <v>343427</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="8" t="n">
         <v>311</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="8" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
+      <c r="A9" s="8" t="n">
         <v>343355</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="8" t="n">
         <v>1710</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="n">
+      <c r="A10" s="8" t="n">
         <v>343355</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="8" t="n">
         <v>569</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="8" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="n">
+      <c r="A11" s="8" t="n">
         <v>343355</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="8" t="n">
         <v>818</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="8" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="n">
+      <c r="A12" s="8" t="n">
         <v>343355</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="8" t="n">
         <v>1481</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="8" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="n">
+      <c r="A13" s="8" t="n">
         <v>343355</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="8" t="n">
         <v>2623</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="n">
+      <c r="A14" s="8" t="n">
         <v>343355</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="8" t="n">
         <v>6256</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="n">
+      <c r="A15" s="8" t="n">
         <v>343428</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="8" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1153,4 +1156,288 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <f aca="false">IF(B6="","",C6-B6)</f>
+        <v>0.0999999999999943</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>1521.7</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>1521.71</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <f aca="false">IF(B7="","",C7-B7)</f>
+        <v>0.00999999999999091</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>68.81</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <f aca="false">IF(B8="","",C8-B8)</f>
+        <v>0.0100000000000051</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>87.1</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <f aca="false">IF(B9="","",C9-B9)</f>
+        <v>0.0999999999999943</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <f aca="false">IF(B10="","",C10-B10)</f>
+        <v>0.0999999999999943</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <f aca="false">IF(B14="","",C14-B14)</f>
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>1519.7</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>1536.34</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <f aca="false">IF(B15="","",C15-B15)</f>
+        <v>16.6399999999999</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>67.27</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <f aca="false">IF(B16="","",C16-B16)</f>
+        <v>-0.730000000000004</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>86.9</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>86.3</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <f aca="false">IF(B17="","",C17-B17)</f>
+        <v>-0.600000000000009</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>72.9</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <f aca="false">IF(B18="","",C18-B18)</f>
+        <v>0.200000000000003</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>41.2</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>66.3</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>295.36</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>287.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A20:C20"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Qwen2.5-VL-7B full results (baseline + BTP) + complete 3-model Excel
</commit_message>
<xml_diff>
--- a/BTP-Reproduction/BTP_Reproduction_Results.xlsx
+++ b/BTP-Reproduction/BTP_Reproduction_Results.xlsx
@@ -11,6 +11,7 @@
     <sheet name="LLaVA-1.5-7B" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Run Log" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="LLaVA-1.5-13B" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Qwen2.5-VL-7B" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="56">
   <si>
     <t xml:space="preserve">BTP Reproduction — LLaVA-v1.5-7B</t>
   </si>
@@ -169,6 +170,27 @@
   </si>
   <si>
     <t xml:space="preserve">IIT Jodhpur HPC, A100-40GB, FlashAttention-2, full datasets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qwen2.5-VL-7B-Instruct — Paper vs Ours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IIT Jodhpur HPC, A100-40GB, FlashAttention-2, full datasets | BTP retention 25%/12.5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BTP (25% / 12.5%) — Paper vs Ours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TextVQA (val)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: SQA — our 88.1/85.1 exceeds paper 76.7/74.1; Qwen2.5-VL is very strong on ScienceQA, likely a prompt/variant difference.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: Full Qwen sweep exceeds 10h SLURM walltime (TIMEOUT on first run); SEED+TextVQA BTP rerun separately.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: SEED/TextVQA BTP on 2000-sample subset. TextVQA-BTP 23.6 (vs baseline 82.7) confirmed across 2 runs - aggressive pruning removes fine-grained tokens needed to read in-image text.</t>
   </si>
 </sst>
 </file>
@@ -179,7 +201,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,6 +257,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -309,8 +337,44 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -326,23 +390,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -601,264 +661,264 @@
   <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="7" t="n">
         <v>62</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <v>61.98</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="7" t="n">
         <f aca="false">C6-B6</f>
         <v>-0.0200000000000031</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <v>1510.7</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="7" t="n">
         <v>1507.5</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="7" t="n">
         <f aca="false">C7-B7</f>
         <v>-3.20000000000005</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="7" t="n">
         <v>64.3</v>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="7" t="n">
         <v>64</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="7" t="n">
         <f aca="false">C8-B8</f>
         <v>-0.299999999999997</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <v>85.8</v>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="7" t="n">
         <v>86.98</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="7" t="n">
         <f aca="false">C9-B9</f>
         <v>1.18000000000001</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>69.4</v>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="7" t="n">
         <v>69.41</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="7" t="n">
         <f aca="false">C10-B10</f>
         <v>0.00999999999999091</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="7" t="n">
         <v>59</v>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="7" t="n">
         <v>58.98</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="7" t="n">
         <f aca="false">C14-B14</f>
         <v>-0.0200000000000031</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="7" t="n">
         <v>1487</v>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="7" t="n">
         <v>1497.2</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D15" s="7" t="n">
         <f aca="false">C15-B15</f>
         <v>10.2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B16" s="7" t="n">
         <v>62.7</v>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="7" t="n">
         <v>63.49</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="7" t="n">
         <f aca="false">C16-B16</f>
         <v>0.789999999999999</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B17" s="7" t="n">
         <v>85.6</v>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="7" t="n">
         <v>85.36</v>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D17" s="7" t="n">
         <f aca="false">C17-B17</f>
         <v>-0.239999999999995</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="6" t="n">
+      <c r="B18" s="7" t="n">
         <v>69.1</v>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="7" t="n">
         <v>69.21</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="7" t="n">
         <f aca="false">C18-B18</f>
         <v>0.109999999999999</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="6" t="n">
+      <c r="B22" s="7" t="n">
         <v>46.11</v>
       </c>
-      <c r="C22" s="6" t="n">
+      <c r="C22" s="7" t="n">
         <v>40.02</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B23" s="6" t="n">
+      <c r="B23" s="7" t="n">
         <v>66.23</v>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C23" s="7" t="n">
         <v>63.99</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="6" t="n">
+      <c r="B24" s="7" t="n">
         <v>355.7</v>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C24" s="7" t="n">
         <v>351.4</v>
       </c>
     </row>
@@ -886,264 +946,264 @@
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="8" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="n">
+      <c r="A2" s="9" t="n">
         <v>343354</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="8" t="n">
+      <c r="D2" s="9" t="n">
         <v>1028</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="9" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="9" t="n">
         <v>343354</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="9" t="n">
         <v>430</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="9" t="n">
         <v>343354</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="9" t="n">
         <v>643</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="9" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="9" t="n">
         <v>343354</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="9" t="n">
         <v>1161</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="9" t="n">
         <v>343354</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="9" t="n">
         <v>2182</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="9" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="9" t="n">
         <v>343354</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <v>9510</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="9" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="9" t="n">
         <v>343427</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="9" t="n">
         <v>311</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="9" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="9" t="n">
         <v>343355</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="9" t="n">
         <v>1710</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="9" t="n">
         <v>343355</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="9" t="n">
         <v>569</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="9" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="n">
+      <c r="A11" s="9" t="n">
         <v>343355</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="9" t="n">
         <v>818</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="9" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
+      <c r="A12" s="9" t="n">
         <v>343355</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="9" t="n">
         <v>1481</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="n">
+      <c r="A13" s="9" t="n">
         <v>343355</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="9" t="n">
         <v>2623</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="9" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
+      <c r="A14" s="9" t="n">
         <v>343355</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="9" t="n">
         <v>6256</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="9" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="n">
+      <c r="A15" s="9" t="n">
         <v>343428</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="9" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1166,263 +1226,263 @@
   <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="7" t="n">
         <v>63.2</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <v>63.3</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="7" t="n">
         <f aca="false">IF(B6="","",C6-B6)</f>
         <v>0.0999999999999943</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <v>1521.7</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="7" t="n">
         <v>1521.71</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="7" t="n">
         <f aca="false">IF(B7="","",C7-B7)</f>
         <v>0.00999999999999091</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="7" t="n">
         <v>68.8</v>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="7" t="n">
         <v>68.81</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="7" t="n">
         <f aca="false">IF(B8="","",C8-B8)</f>
         <v>0.0100000000000051</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <v>87</v>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="7" t="n">
         <v>87.1</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="7" t="n">
         <f aca="false">IF(B9="","",C9-B9)</f>
         <v>0.0999999999999943</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>72.7</v>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="7" t="n">
         <v>72.8</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="7" t="n">
         <f aca="false">IF(B10="","",C10-B10)</f>
         <v>0.0999999999999943</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="7" t="n">
         <v>62.2</v>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="7" t="n">
         <v>60.7</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="7" t="n">
         <f aca="false">IF(B14="","",C14-B14)</f>
         <v>-1.5</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="7" t="n">
         <v>1519.7</v>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="7" t="n">
         <v>1536.34</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D15" s="7" t="n">
         <f aca="false">IF(B15="","",C15-B15)</f>
         <v>16.6399999999999</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B16" s="7" t="n">
         <v>68</v>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="7" t="n">
         <v>67.27</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="7" t="n">
         <f aca="false">IF(B16="","",C16-B16)</f>
         <v>-0.730000000000004</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B17" s="7" t="n">
         <v>86.9</v>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="7" t="n">
         <v>86.3</v>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D17" s="7" t="n">
         <f aca="false">IF(B17="","",C17-B17)</f>
         <v>-0.600000000000009</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="6" t="n">
+      <c r="B18" s="7" t="n">
         <v>72.7</v>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="7" t="n">
         <v>72.9</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="7" t="n">
         <f aca="false">IF(B18="","",C18-B18)</f>
         <v>0.200000000000003</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="6" t="n">
+      <c r="B22" s="7" t="n">
         <v>48.8</v>
       </c>
-      <c r="C22" s="6" t="n">
+      <c r="C22" s="7" t="n">
         <v>41.2</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B23" s="6" t="n">
+      <c r="B23" s="7" t="n">
         <v>68.2</v>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C23" s="7" t="n">
         <v>66.3</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="6" t="n">
+      <c r="B24" s="7" t="n">
         <v>295.36</v>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C24" s="7" t="n">
         <v>287.5</v>
       </c>
     </row>
@@ -1440,4 +1500,315 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="D6" s="14" t="n">
+        <f aca="false">C6-B6</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>1690.8</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>1674.47</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <f aca="false">C7-B7</f>
+        <v>-16.3299999999999</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>83.68</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <f aca="false">C8-B8</f>
+        <v>1.18000000000001</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>87.4</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>87.6</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <f aca="false">C9-B9</f>
+        <v>0.199999999999989</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>88.1</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <f aca="false">C10-B10</f>
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <f aca="false">C14-B14</f>
+        <v>-1.3</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>1651.5</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1658.67</v>
+      </c>
+      <c r="D15" s="14" t="n">
+        <f aca="false">C15-B15</f>
+        <v>7.17000000000007</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <f aca="false">C16-B16</f>
+        <v>4.09999999999999</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>86.2</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>86.2</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <f aca="false">C17-B17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>74.1</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>85.1</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <f aca="false">C18-B18</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>82.7</v>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>23.6</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>73.1</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>618.57</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>557.14</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A28:D28"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>